<commit_message>
Limit share of voice file to the requested retailers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RzXUNWe52FPe7pzHpD5YVj
</commit_message>
<xml_diff>
--- a/Meta_share_of_voice_by_retailer.xlsx
+++ b/Meta_share_of_voice_by_retailer.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Share of voice'!$A$1:$F$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Share of voice'!$A$1:$F$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -770,19 +770,19 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>John-Lewis</t>
+          <t>BestBuy-US</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -791,21 +791,21 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.457</v>
+        <v>0.711</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.506</v>
+        <v>0.773</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C11" s="6" t="n"/>
@@ -815,26 +815,26 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.442</v>
+        <v>0.542</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.464</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>O2-GB</t>
+          <t>Amazon-US</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -842,24 +842,22 @@
           <t>Wearables</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E12" s="5" t="n">
+        <v>0.374</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.218</v>
+        <v>0.407</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C13" s="6" t="n"/>
@@ -868,29 +866,27 @@
           <t>VR</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E13" s="5" t="n">
+        <v>0.349</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.357</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Very-UK</t>
+          <t>Walmart-US</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -899,21 +895,21 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0</v>
+        <v>0.422</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.489</v>
+        <v>0.456</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
@@ -923,26 +919,26 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0</v>
+        <v>0.386</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.342</v>
+        <v>0.459</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Amazon-DE</t>
+          <t>Target-US</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -951,21 +947,21 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.256</v>
+        <v>0.578</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.182</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C17" s="6" t="n"/>
@@ -975,26 +971,26 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.26</v>
+        <v>0.48</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.271</v>
+        <v>0.603</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Alternate-DE</t>
+          <t>Verizon-US</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1003,21 +999,21 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0</v>
+        <v>0.774</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0</v>
+        <v>0.785</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C19" s="6" t="n"/>
@@ -1027,26 +1023,26 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.53</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.611</v>
+        <v>0.5870000000000001</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Freenet-DE</t>
+          <t>APP: Amazon-US</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1055,21 +1051,21 @@
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.377</v>
+        <v>0.304</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.404</v>
+        <v>0.304</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
@@ -1079,26 +1075,26 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.186</v>
+        <v>0.335</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.183</v>
+        <v>0.335</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Media-Markt-DE</t>
+          <t>APP: BestBuy-US</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -1107,21 +1103,21 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.318</v>
+        <v>0.631</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.314</v>
+        <v>0.631</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
@@ -1131,26 +1127,26 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.221</v>
+        <v>0.368</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.252</v>
+        <v>0.368</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Telefonica-DE</t>
+          <t>APP: Walmart-US</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -1159,21 +1155,21 @@
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.076</v>
+        <v>0.315</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.305</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C25" s="6" t="n"/>
@@ -1183,26 +1179,26 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.449</v>
+        <v>0.494</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.67</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Amazon-FR</t>
+          <t>APP: Target-US</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -1211,21 +1207,21 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.271</v>
+        <v>0.5820000000000001</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.211</v>
+        <v>0.5820000000000001</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C27" s="6" t="n"/>
@@ -1235,26 +1231,26 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>0.331</v>
+        <v>0.255</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.354</v>
+        <v>0.255</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Boulanger-FR</t>
+          <t>Amazon-CA</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1263,21 +1259,21 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.636</v>
+        <v>0.384</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.6509999999999999</v>
+        <v>0.393</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C29" s="6" t="n"/>
@@ -1287,26 +1283,26 @@
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>0.238</v>
+        <v>0.329</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.231</v>
+        <v>0.344</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>FNAC-FR</t>
+          <t>BestBuy-CA</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1315,21 +1311,21 @@
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.511</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.604</v>
+        <v>0.517</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C31" s="6" t="n"/>
@@ -1339,26 +1335,26 @@
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.355</v>
+        <v>0.503</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.364</v>
+        <v>0.413</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>SFR-FR</t>
+          <t>Walmart-CA</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -1367,21 +1363,21 @@
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.073</v>
+        <v>0.38</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.091</v>
+        <v>0.347</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Meta Americas</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C33" s="6" t="n"/>
@@ -1391,26 +1387,26 @@
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>0</v>
+        <v>0.5429999999999999</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0</v>
+        <v>0.508</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Amazon-ES</t>
+          <t>JB-HiFi-AU</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -1419,21 +1415,21 @@
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.242</v>
+        <v>0.54</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.17</v>
+        <v>0.7290000000000001</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C35" s="6" t="n"/>
@@ -1443,26 +1439,26 @@
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>0.267</v>
+        <v>0.524</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.303</v>
+        <v>0.534</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Elcorteingles-Store-ES</t>
+          <t>Telstra-AU</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1471,21 +1467,21 @@
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.143</v>
+        <v>0.249</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.172</v>
+        <v>0.249</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C37" s="6" t="n"/>
@@ -1495,10 +1491,10 @@
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>0.266</v>
+        <v>0.001</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.298</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="38">
@@ -1509,12 +1505,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>MediaMarkt-ES</t>
+          <t>Media-Markt-DE</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1523,10 +1519,10 @@
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.356</v>
+        <v>0.318</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.482</v>
+        <v>0.314</v>
       </c>
     </row>
     <row r="39">
@@ -1537,7 +1533,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C39" s="6" t="n"/>
@@ -1547,10 +1543,10 @@
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>0.136</v>
+        <v>0.221</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.155</v>
+        <v>0.252</v>
       </c>
     </row>
     <row r="40">
@@ -1561,12 +1557,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Movistar-ES</t>
+          <t>Deutsche Telekom DE</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1579,8 +1575,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F40" s="5" t="n">
-        <v>0.479</v>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1591,7 +1589,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C41" s="6" t="n"/>
@@ -1605,8 +1603,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F41" s="5" t="n">
-        <v>0.245</v>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -1617,12 +1617,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Orange-ES</t>
+          <t>FNAC-FR</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -1630,13 +1630,11 @@
           <t>Wearables</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E42" s="5" t="n">
+        <v>0.5570000000000001</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.626</v>
+        <v>0.604</v>
       </c>
     </row>
     <row r="43">
@@ -1647,7 +1645,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C43" s="6" t="n"/>
@@ -1656,29 +1654,27 @@
           <t>VR</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E43" s="5" t="n">
+        <v>0.355</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.227</v>
+        <v>0.364</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Elkjop-NO</t>
+          <t>Amazon-JP</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -1687,21 +1683,21 @@
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>0.353</v>
+        <v>0.155</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.338</v>
+        <v>0.236</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C45" s="6" t="n"/>
@@ -1711,26 +1707,26 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>0.136</v>
+        <v>0.091</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.13</v>
+        <v>0.052</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Elkjop-SE</t>
+          <t>Yodobashi-JP</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -1739,21 +1735,21 @@
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>0.321</v>
+        <v>0.203</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.321</v>
+        <v>0.203</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C47" s="6" t="n"/>
@@ -1763,26 +1759,26 @@
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>0.207</v>
+        <v>0.133</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.189</v>
+        <v>0.133</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Komplett-SE</t>
+          <t>BIC-JP</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -1790,26 +1786,22 @@
           <t>Wearables</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E48" s="5" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>0.129</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Meta Western Europe</t>
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C49" s="6" t="n"/>
@@ -1819,26 +1811,26 @@
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>0.299</v>
+        <v>0.077</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0.385</v>
+        <v>0.065</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>ATT-US</t>
+          <t>Softbank JP</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -1846,22 +1838,26 @@
           <t>Wearables</t>
         </is>
       </c>
-      <c r="E50" s="5" t="n">
-        <v>0.504</v>
-      </c>
-      <c r="F50" s="5" t="n">
-        <v>0.496</v>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C51" s="6" t="n"/>
@@ -1870,27 +1866,31 @@
           <t>VR</t>
         </is>
       </c>
-      <c r="E51" s="5" t="n">
-        <v>0.251</v>
-      </c>
-      <c r="F51" s="5" t="n">
-        <v>0.332</v>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Meta Western Europe</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Amazon-US</t>
+          <t>Elkjop-NO</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -1899,21 +1899,21 @@
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>0.374</v>
+        <v>0.353</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.407</v>
+        <v>0.338</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Meta Western Europe</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="C53" s="6" t="n"/>
@@ -1923,10 +1923,10 @@
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>0.349</v>
+        <v>0.136</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0.357</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="54">
@@ -1937,12 +1937,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>APP: Amazon-US</t>
+          <t>Amazon-MX</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>0.304</v>
+        <v>0.184</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>0.304</v>
+        <v>0.159</v>
       </c>
     </row>
     <row r="55">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C55" s="6" t="n"/>
@@ -1975,26 +1975,26 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>0.335</v>
+        <v>0.19</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>0.335</v>
+        <v>0.229</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>BestBuy-US</t>
+          <t>Amazon-IN</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -2003,21 +2003,21 @@
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>0.711</v>
+        <v>0.285</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>0.773</v>
+        <v>0.249</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C57" s="6" t="n"/>
@@ -2027,26 +2027,26 @@
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>0.542</v>
+        <v>0.18</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>0.63</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>APP: BestBuy-US</t>
+          <t>Flipkart-IN</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2055,21 +2055,21 @@
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>0.631</v>
+        <v>0.096</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>0.631</v>
+        <v>0.108</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C59" s="6" t="n"/>
@@ -2079,26 +2079,26 @@
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>0.368</v>
+        <v>0.326</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>0.368</v>
+        <v>0.471</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>TMobile-US</t>
+          <t>APP: Flipkart-IN</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -2107,21 +2107,21 @@
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>0.5539999999999999</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>0.57</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>Meta APAC</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C61" s="6" t="n"/>
@@ -2131,26 +2131,26 @@
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>0.4320000000000001</v>
+        <v>0.225</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>0.575</v>
+        <v>0.225</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Meta Western Europe</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Target-US</t>
+          <t>Movistar-ES</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -2158,22 +2158,24 @@
           <t>Wearables</t>
         </is>
       </c>
-      <c r="E62" s="5" t="n">
-        <v>0.578</v>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0.485</v>
+        <v>0.479</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Meta Western Europe</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C63" s="6" t="n"/>
@@ -2182,1054 +2184,49 @@
           <t>VR</t>
         </is>
       </c>
-      <c r="E63" s="5" t="n">
-        <v>0.48</v>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F63" s="5" t="n">
-        <v>0.603</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>APP: Target-US</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E64" s="5" t="n">
-        <v>0.5820000000000001</v>
-      </c>
-      <c r="F64" s="5" t="n">
-        <v>0.5820000000000001</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C65" s="6" t="n"/>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="n">
-        <v>0.255</v>
-      </c>
-      <c r="F65" s="5" t="n">
-        <v>0.255</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>Verizon-US</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="n">
-        <v>0.774</v>
-      </c>
-      <c r="F66" s="5" t="n">
-        <v>0.785</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C67" s="6" t="n"/>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="F67" s="5" t="n">
-        <v>0.5870000000000001</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Walmart-US</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="n">
-        <v>0.422</v>
-      </c>
-      <c r="F68" s="5" t="n">
-        <v>0.456</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C69" s="6" t="n"/>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="n">
-        <v>0.386</v>
-      </c>
-      <c r="F69" s="5" t="n">
-        <v>0.459</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>APP: Walmart-US</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="n">
-        <v>0.315</v>
-      </c>
-      <c r="F70" s="5" t="n">
-        <v>0.305</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="n"/>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="n">
-        <v>0.494</v>
-      </c>
-      <c r="F71" s="5" t="n">
-        <v>0.48</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>Amazon-CA</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="n">
-        <v>0.384</v>
-      </c>
-      <c r="F72" s="5" t="n">
-        <v>0.393</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="n"/>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="n">
-        <v>0.329</v>
-      </c>
-      <c r="F73" s="5" t="n">
-        <v>0.344</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>BestBuy-CA</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="n">
-        <v>0.511</v>
-      </c>
-      <c r="F74" s="5" t="n">
-        <v>0.517</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="C75" s="6" t="n"/>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E75" s="5" t="n">
-        <v>0.503</v>
-      </c>
-      <c r="F75" s="5" t="n">
-        <v>0.413</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>Walmart-CA</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E76" s="5" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="F76" s="5" t="n">
-        <v>0.347</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="C77" s="6" t="n"/>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E77" s="5" t="n">
-        <v>0.5429999999999999</v>
-      </c>
-      <c r="F77" s="5" t="n">
-        <v>0.508</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>Amazon-MX</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="n">
-        <v>0.184</v>
-      </c>
-      <c r="F78" s="5" t="n">
-        <v>0.159</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="7" t="inlineStr">
-        <is>
-          <t>Meta Americas</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="n"/>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="F79" s="5" t="n">
-        <v>0.229</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>Amazon-AU</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="n">
-        <v>0.336</v>
-      </c>
-      <c r="F80" s="5" t="n">
-        <v>0.329</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="n"/>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="n">
-        <v>0.252</v>
-      </c>
-      <c r="F81" s="5" t="n">
-        <v>0.291</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
-        <is>
-          <t>Harvey-Norman-AU</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="n">
-        <v>0.478</v>
-      </c>
-      <c r="F82" s="5" t="n">
-        <v>0.632</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C83" s="6" t="n"/>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="n">
-        <v>0.4970000000000001</v>
-      </c>
-      <c r="F83" s="5" t="n">
-        <v>0.444</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C84" s="4" t="inlineStr">
-        <is>
-          <t>JB-HiFi-AU</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="F84" s="5" t="n">
-        <v>0.7290000000000001</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C85" s="6" t="n"/>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E85" s="5" t="n">
-        <v>0.524</v>
-      </c>
-      <c r="F85" s="5" t="n">
-        <v>0.534</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C86" s="4" t="inlineStr">
-        <is>
-          <t>Telstra-AU</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E86" s="5" t="n">
-        <v>0.249</v>
-      </c>
-      <c r="F86" s="5" t="n">
-        <v>0.249</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B87" s="3" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="n"/>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="F87" s="5" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C88" s="4" t="inlineStr">
-        <is>
-          <t>Amazon-JP</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="n">
-        <v>0.155</v>
-      </c>
-      <c r="F88" s="5" t="n">
-        <v>0.236</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C89" s="6" t="n"/>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E89" s="5" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="F89" s="5" t="n">
-        <v>0.052</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B90" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C90" s="4" t="inlineStr">
-        <is>
-          <t>BIC-JP</t>
-        </is>
-      </c>
-      <c r="D90" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="F90" s="5" t="n">
-        <v>0.129</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C91" s="6" t="n"/>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E91" s="5" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="F91" s="5" t="n">
-        <v>0.065</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B92" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>Yamada-Denki-JP</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F92" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="n"/>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E93" s="5" t="n">
-        <v>0.183</v>
-      </c>
-      <c r="F93" s="5" t="n">
-        <v>0.079</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B94" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C94" s="4" t="inlineStr">
-        <is>
-          <t>Yodobashi-JP</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="n">
-        <v>0.203</v>
-      </c>
-      <c r="F94" s="5" t="n">
-        <v>0.203</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="C95" s="6" t="n"/>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="n">
-        <v>0.133</v>
-      </c>
-      <c r="F95" s="5" t="n">
-        <v>0.133</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B96" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="C96" s="4" t="inlineStr">
-        <is>
-          <t>Amazon-IN</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E96" s="5" t="n">
-        <v>0.285</v>
-      </c>
-      <c r="F96" s="5" t="n">
-        <v>0.249</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B97" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="C97" s="6" t="n"/>
-      <c r="D97" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E97" s="5" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="F97" s="5" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B98" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="C98" s="4" t="inlineStr">
-        <is>
-          <t>Flipkart-IN</t>
-        </is>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="n">
-        <v>0.096</v>
-      </c>
-      <c r="F98" s="5" t="n">
-        <v>0.108</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B99" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="C99" s="6" t="n"/>
-      <c r="D99" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E99" s="5" t="n">
-        <v>0.326</v>
-      </c>
-      <c r="F99" s="5" t="n">
-        <v>0.471</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B100" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="C100" s="4" t="inlineStr">
-        <is>
-          <t>APP: Flipkart-IN</t>
-        </is>
-      </c>
-      <c r="D100" s="3" t="inlineStr">
-        <is>
-          <t>Wearables</t>
-        </is>
-      </c>
-      <c r="E100" s="5" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-      <c r="F100" s="5" t="n">
-        <v>0.08599999999999999</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="8" t="inlineStr">
-        <is>
-          <t>Meta APAC</t>
-        </is>
-      </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="C101" s="6" t="n"/>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>VR</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="n">
-        <v>0.225</v>
-      </c>
-      <c r="F101" s="5" t="n">
-        <v>0.225</v>
+        <v>0.245</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F101"/>
-  <mergeCells count="50">
+  <autoFilter ref="A1:F63"/>
+  <mergeCells count="31">
     <mergeCell ref="C30:C31"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="C42:C43"/>
     <mergeCell ref="C20:C21"/>
-    <mergeCell ref="C94:C95"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="C54:C55"/>
     <mergeCell ref="C50:C51"/>
-    <mergeCell ref="C88:C89"/>
     <mergeCell ref="C26:C27"/>
     <mergeCell ref="C44:C45"/>
-    <mergeCell ref="C84:C85"/>
     <mergeCell ref="C22:C23"/>
-    <mergeCell ref="C100:C101"/>
-    <mergeCell ref="C80:C81"/>
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="C56:C57"/>
-    <mergeCell ref="C90:C91"/>
     <mergeCell ref="C46:C47"/>
     <mergeCell ref="C58:C59"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="C36:C37"/>
-    <mergeCell ref="C76:C77"/>
     <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C70:C71"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="C60:C61"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="C82:C83"/>
-    <mergeCell ref="C72:C73"/>
-    <mergeCell ref="C78:C79"/>
     <mergeCell ref="C32:C33"/>
-    <mergeCell ref="C96:C97"/>
     <mergeCell ref="C48:C49"/>
-    <mergeCell ref="C86:C87"/>
     <mergeCell ref="C62:C63"/>
     <mergeCell ref="C38:C39"/>
     <mergeCell ref="C34:C35"/>
     <mergeCell ref="C28:C29"/>
-    <mergeCell ref="C74:C75"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="C64:C65"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="C24:C25"/>
     <mergeCell ref="C18:C19"/>
     <mergeCell ref="C14:C15"/>
-    <mergeCell ref="C98:C99"/>
-    <mergeCell ref="C92:C93"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3285,7 +2282,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Retailers with partial history (e.g. Telstra from Sep 3, Elkjop SE ended Aug 27, app retailers from Aug) have shorter windows than the headers say.</t>
+          <t>Deutsche Telekom DE and Softbank JP are not in the Meta scorecards (no data). Retailers with partial history (e.g. Telstra from Sep 3, Elkjop SE ended Aug 27, app retailers from Aug) have shorter windows than the headers say.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use platform's weighted search terms for share of voice
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RzXUNWe52FPe7pzHpD5YVj
</commit_message>
<xml_diff>
--- a/Meta_share_of_voice_by_retailer.xlsx
+++ b/Meta_share_of_voice_by_retailer.xlsx
@@ -579,10 +579,10 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.59</v>
+        <v>0.6978</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.67</v>
+        <v>0.6737000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.322</v>
+        <v>0.3129</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.301</v>
+        <v>0.2939</v>
       </c>
     </row>
     <row r="4">
@@ -631,10 +631,10 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.83</v>
+        <v>0.8096</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.8390000000000001</v>
+        <v>0.7655</v>
       </c>
     </row>
     <row r="5">
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.667</v>
+        <v>0.6801999999999999</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.633</v>
+        <v>0.6101</v>
       </c>
     </row>
     <row r="6">
@@ -683,10 +683,10 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.393</v>
+        <v>0.5745</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.344</v>
+        <v>0.383</v>
       </c>
     </row>
     <row r="7">
@@ -707,10 +707,10 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.289</v>
+        <v>0.3927</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.308</v>
+        <v>0.3599</v>
       </c>
     </row>
     <row r="8">
@@ -791,10 +791,10 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.711</v>
+        <v>0.8509</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.773</v>
+        <v>0.8578</v>
       </c>
     </row>
     <row r="11">
@@ -815,10 +815,10 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.542</v>
+        <v>0.6327</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.63</v>
+        <v>0.6368</v>
       </c>
     </row>
     <row r="12">
@@ -843,10 +843,10 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.374</v>
+        <v>0.5549000000000001</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.407</v>
+        <v>0.5676</v>
       </c>
     </row>
     <row r="13">
@@ -867,10 +867,10 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.349</v>
+        <v>0.4776</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.357</v>
+        <v>0.4727</v>
       </c>
     </row>
     <row r="14">
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.422</v>
+        <v>0.6163000000000001</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.456</v>
+        <v>0.5623</v>
       </c>
     </row>
     <row r="15">
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.386</v>
+        <v>0.5435</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.459</v>
+        <v>0.5757</v>
       </c>
     </row>
     <row r="16">
@@ -947,10 +947,10 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.578</v>
+        <v>0.6893</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.485</v>
+        <v>0.5891</v>
       </c>
     </row>
     <row r="17">
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.48</v>
+        <v>0.4884000000000001</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.603</v>
+        <v>0.575</v>
       </c>
     </row>
     <row r="18">
@@ -999,10 +999,10 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.774</v>
+        <v>0.7315</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.785</v>
+        <v>0.7363</v>
       </c>
     </row>
     <row r="19">
@@ -1023,10 +1023,10 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.53</v>
+        <v>0.5415</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.5870000000000001</v>
+        <v>0.5579</v>
       </c>
     </row>
     <row r="20">
@@ -1051,10 +1051,10 @@
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.304</v>
+        <v>0.4328</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.304</v>
+        <v>0.4328</v>
       </c>
     </row>
     <row r="21">
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.335</v>
+        <v>0.4839</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.335</v>
+        <v>0.4839</v>
       </c>
     </row>
     <row r="22">
@@ -1103,10 +1103,10 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.631</v>
+        <v>0.7831</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.631</v>
+        <v>0.7831</v>
       </c>
     </row>
     <row r="23">
@@ -1127,10 +1127,10 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.368</v>
+        <v>0.4757</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.368</v>
+        <v>0.4757</v>
       </c>
     </row>
     <row r="24">
@@ -1155,10 +1155,10 @@
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.315</v>
+        <v>0.5182</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.305</v>
+        <v>0.4679</v>
       </c>
     </row>
     <row r="25">
@@ -1179,10 +1179,10 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.494</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.48</v>
+        <v>0.5145000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1207,10 +1207,10 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.5820000000000001</v>
+        <v>0.7291</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.5820000000000001</v>
+        <v>0.7291</v>
       </c>
     </row>
     <row r="27">
@@ -1231,10 +1231,10 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>0.255</v>
+        <v>0.2871</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.255</v>
+        <v>0.2871</v>
       </c>
     </row>
     <row r="28">
@@ -1259,10 +1259,10 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.384</v>
+        <v>0.5561</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.393</v>
+        <v>0.5297999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -1283,10 +1283,10 @@
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>0.329</v>
+        <v>0.4705</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.344</v>
+        <v>0.4425</v>
       </c>
     </row>
     <row r="30">
@@ -1311,10 +1311,10 @@
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.511</v>
+        <v>0.638</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.517</v>
+        <v>0.623</v>
       </c>
     </row>
     <row r="31">
@@ -1335,10 +1335,10 @@
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.503</v>
+        <v>0.5536</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.413</v>
+        <v>0.4549</v>
       </c>
     </row>
     <row r="32">
@@ -1363,10 +1363,10 @@
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.38</v>
+        <v>0.5132</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.347</v>
+        <v>0.3612</v>
       </c>
     </row>
     <row r="33">
@@ -1387,10 +1387,10 @@
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>0.5429999999999999</v>
+        <v>0.5949</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.508</v>
+        <v>0.5274</v>
       </c>
     </row>
     <row r="34">
@@ -1415,10 +1415,10 @@
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.54</v>
+        <v>0.645</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.7290000000000001</v>
+        <v>0.7519</v>
       </c>
     </row>
     <row r="35">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>0.524</v>
+        <v>0.5272</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.534</v>
+        <v>0.4935</v>
       </c>
     </row>
     <row r="36">
@@ -1467,10 +1467,10 @@
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.249</v>
+        <v>0.4686</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.249</v>
+        <v>0.4686</v>
       </c>
     </row>
     <row r="37">
@@ -1491,10 +1491,10 @@
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="38">
@@ -1519,10 +1519,10 @@
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.318</v>
+        <v>0.3534</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.314</v>
+        <v>0.2716</v>
       </c>
     </row>
     <row r="39">
@@ -1543,10 +1543,10 @@
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>0.221</v>
+        <v>0.2783</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.252</v>
+        <v>0.1972</v>
       </c>
     </row>
     <row r="40">
@@ -1631,10 +1631,10 @@
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5426</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.604</v>
+        <v>0.5645</v>
       </c>
     </row>
     <row r="43">
@@ -1655,10 +1655,10 @@
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>0.355</v>
+        <v>0.3395</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.364</v>
+        <v>0.3327000000000001</v>
       </c>
     </row>
     <row r="44">
@@ -1683,10 +1683,10 @@
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>0.155</v>
+        <v>0.1274</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.236</v>
+        <v>0.2197</v>
       </c>
     </row>
     <row r="45">
@@ -1707,10 +1707,10 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>0.091</v>
+        <v>0.0248</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.052</v>
+        <v>0.0238</v>
       </c>
     </row>
     <row r="46">
@@ -1735,10 +1735,10 @@
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>0.203</v>
+        <v>0.1698</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.203</v>
+        <v>0.1698</v>
       </c>
     </row>
     <row r="47">
@@ -1759,10 +1759,10 @@
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>0.133</v>
+        <v>0.03</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.133</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="48">
@@ -1787,10 +1787,10 @@
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>0.128</v>
+        <v>0.07870000000000001</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>0.129</v>
+        <v>0.08220000000000001</v>
       </c>
     </row>
     <row r="49">
@@ -1811,10 +1811,10 @@
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>0.077</v>
+        <v>0.0144</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0.065</v>
+        <v>0.0363</v>
       </c>
     </row>
     <row r="50">
@@ -1899,10 +1899,10 @@
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>0.353</v>
+        <v>0.3948</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.338</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="53">
@@ -1923,10 +1923,10 @@
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>0.136</v>
+        <v>0.1052</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0.13</v>
+        <v>0.09269999999999999</v>
       </c>
     </row>
     <row r="54">
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>0.184</v>
+        <v>0.1832</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>0.159</v>
+        <v>0.1418</v>
       </c>
     </row>
     <row r="55">
@@ -1975,10 +1975,10 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>0.19</v>
+        <v>0.2597</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>0.229</v>
+        <v>0.2669</v>
       </c>
     </row>
     <row r="56">
@@ -2003,10 +2003,10 @@
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>0.285</v>
+        <v>0.2808</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>0.249</v>
+        <v>0.2508</v>
       </c>
     </row>
     <row r="57">
@@ -2027,10 +2027,10 @@
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>0.18</v>
+        <v>0.09449999999999999</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>0.28</v>
+        <v>0.1002</v>
       </c>
     </row>
     <row r="58">
@@ -2055,10 +2055,10 @@
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>0.096</v>
+        <v>0.09470000000000001</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>0.108</v>
+        <v>0.1074</v>
       </c>
     </row>
     <row r="59">
@@ -2079,10 +2079,10 @@
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>0.326</v>
+        <v>0.2784</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>0.471</v>
+        <v>0.3044</v>
       </c>
     </row>
     <row r="60">
@@ -2107,10 +2107,10 @@
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08380000000000001</v>
       </c>
       <c r="F60" s="5" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08380000000000001</v>
       </c>
     </row>
     <row r="61">
@@ -2131,10 +2131,10 @@
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>0.225</v>
+        <v>0.2323</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>0.225</v>
+        <v>0.2323</v>
       </c>
     </row>
     <row r="62">
@@ -2164,7 +2164,7 @@
         </is>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0.479</v>
+        <v>0.4924</v>
       </c>
     </row>
     <row r="63">
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="F63" s="5" t="n">
-        <v>0.245</v>
+        <v>0.2622</v>
       </c>
     </row>
   </sheetData>
@@ -2261,7 +2261,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Method: score summed per search term per day (client brands), then averaged across all term-days in the period.</t>
+          <t>Method: score summed per search term per day (client brands), then averaged across term-days for the search terms with a search-term weight set (the terms the platform scores). Matches the platform for Best Buy US VR (63.68%) and Target US VR (57.50%) YTD.</t>
         </is>
       </c>
     </row>

</xml_diff>